<commit_message>
data(q2): refresh Origin package and preserve old data
</commit_message>
<xml_diff>
--- a/modules/30_q2/figures/editable/origin_templates/data_package/09_厚度结果柱状图.xlsx
+++ b/modules/30_q2/figures/editable/origin_templates/data_package/09_厚度结果柱状图.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_厚度结果柱状图" sheetId="1" r:id="R2275ed54c3dc497f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_厚度结果柱状图" sheetId="1" r:id="Rdcc8a9d0fc004857"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19,15 +19,15 @@
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
-      <x:sz val="10"/>
+      <x:sz val="11"/>
       <x:color rgb="FF222222"/>
-      <x:name val="Microsoft YaHei"/>
+      <x:name val="Carlito"/>
     </x:font>
     <x:font>
       <x:b/>
-      <x:sz val="10"/>
+      <x:sz val="11"/>
       <x:color rgb="FFFFFFFF"/>
-      <x:name val="Microsoft YaHei"/>
+      <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
   <x:fills count="3">
@@ -63,24 +63,18 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="9">
+  <x:cellXfs count="7">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -283,48 +277,40 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="12.25" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="10.75" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="34" customHeight="1">
-      <x:c r="A1" s="7" t="str">
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="6" t="str">
         <x:v>厚度结果-X</x:v>
       </x:c>
-      <x:c r="B1" s="7" t="str">
+      <x:c r="B1" s="6" t="str">
         <x:v>厚度(微米)-Y</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="8" t="str">
+      <x:c r="A2" s="2" t="str">
         <x:v>10度单角度</x:v>
       </x:c>
-      <x:c r="B2" s="8" t="n">
-        <x:v>7.85663582063064</x:v>
+      <x:c r="B2" s="2" t="n">
+        <x:v>7.856635820616846</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="8" t="str">
+      <x:c r="A3" s="2" t="str">
         <x:v>15度单角度</x:v>
       </x:c>
-      <x:c r="B3" s="8" t="n">
-        <x:v>7.622957415207603</x:v>
+      <x:c r="B3" s="2" t="n">
+        <x:v>7.622957415253701</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="8" t="str">
+      <x:c r="A4" s="2" t="str">
         <x:v>单角度平均</x:v>
       </x:c>
-      <x:c r="B4" s="8" t="n">
-        <x:v>7.739796617919121</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="8" t="str">
-        <x:v>双角度联合验证</x:v>
-      </x:c>
-      <x:c r="B5" s="8" t="n">
-        <x:v>7.739015675125983</x:v>
+      <x:c r="B4" s="2" t="n">
+        <x:v>7.739796617935274</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>